<commit_message>
Bump the parish-meeting layout revision after the table grew
The saved-layout table gained the tower and roofline strand moves after
revision 4, so a layout migrated at revision 4 would miss them. Revision
5 runs the (idempotent) migration once more. Exports, registers and the
safety review refreshed for the stored setting.

Checks: build_parish_migration --check current; --electrical
--export-electrical, register workflow, safety review --check passed.
Web: prepare-viewer, check:viewer (72 files, exact) and check:boundary
(no failures); visit-only mode loads with the Simulator panel hidden.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/electrical-grid/categories/air-system/register.xlsx
+++ b/docs/electrical-grid/categories/air-system/register.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R9efe0ad8efd7406d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rb850016c60604df4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Electrical Lines" sheetId="3" r:id="R1954c5ae925c43d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Points" sheetId="4" r:id="Rc43ec3a575cc4786"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R4ee5a53728384111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R1b6fb52a3a074e00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Electrical Lines" sheetId="3" r:id="R39214289c12c4832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Points" sheetId="4" r:id="Rf734f7aea25e44b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -493,7 +493,7 @@
         <x:v>Baseline</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>Fans and ventilation. Ceiling, wall, entrance and exhaust fans for air movement and ventilation. Model snapshot: 2026-10-24T18:07:55.978Z.</x:v>
+        <x:v>Fans and ventilation. Ceiling, wall, entrance and exhaust fans for air movement and ventilation. Model snapshot: 2026-10-24T18:15:14.532Z.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -576,7 +576,7 @@
         <x:v>Source layout SHA-256</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>5385d4f4cf361a2e56db9b88d4a9952e6d93bf5f83f0834cb083bcdd6684e517</x:v>
+        <x:v>944ecbe81a903e81a65ffa487f20c3a417603b0749843148bbf77414d42d60b4</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="44" customHeight="1">
@@ -4356,7 +4356,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra525fc5b7d8a4b8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1d407e7756a4717"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8975,7 +8975,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae1a096c90d455d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd265785bb79d4d1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20067,7 +20067,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75c4dd1022c4b00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a9968331c894f20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>